<commit_message>
Remove redundant code cardinality comment cbee8e3fdb48ea3f13789505ddc35df200466b81
</commit_message>
<xml_diff>
--- a/nr-doc-core-allergy-intolerance/ig/StructureDefinition-fr-core-practitioner.xlsx
+++ b/nr-doc-core-allergy-intolerance/ig/StructureDefinition-fr-core-practitioner.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-03T09:32:19+00:00</t>
+    <t>2026-09-16T08:22:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1561,7 +1561,7 @@
     <t>Practitioner.qualification:degree.code.coding:degree</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J105-EnsembleDiplome-RASS/FHIR/JDV-J105-EnsembleDiplome-RASS|20260223120000</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J105-EnsembleDiplome-RASS/FHIR/JDV-J105-EnsembleDiplome-RASS|20260730120000</t>
   </si>
   <si>
     <t>Practitioner.qualification:degree.code.text</t>
@@ -1715,7 +1715,7 @@
     <t>Compétence acquise par le professionnel (competence) R39 ou Compétence exclusive exercée par le professionnel à titre exclusif (competenceExclusive) R40 ou Diplôme d'études spécialisées complémentaires (DESC)DESCnonQualifian R42 ou Capacité (savoir-faire)de médecine (capaciteSavoirFaire) R43 ou Qualification de praticien adjoint contractuel (qualificationPAC) R44 ou Fonction qualifiée (Synonyme: fonctionQualifiee) R45 ou Droit d'exercice complémentaire (Synonyme: droitExerciceComplementaire) R97 ou Orientation particulière (Synonyme: orientationParticuliere) G13 ou Activité ponctuelle du professionnel de type expertise (attributionParticuliere) G13.</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J107-EnsembleSavoirFaire-RASS/FHIR/JDV-J107-EnsembleSavoirFaire-RASS|20251222120000</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J107-EnsembleSavoirFaire-RASS/FHIR/JDV-J107-EnsembleSavoirFaire-RASS|20260730120000</t>
   </si>
   <si>
     <t>Practitioner.qualification:savoirFaire.code.text</t>

</xml_diff>